<commit_message>
Time Logs - Final Code
</commit_message>
<xml_diff>
--- a/Issue Tracker v2/gitlab_time_logs.xlsx
+++ b/Issue Tracker v2/gitlab_time_logs.xlsx
@@ -458,7 +458,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -466,11 +466,11 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2025-12-16 15:10:20</t>
+          <t>2025-12-09 16:13:28</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -492,11 +492,11 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.03</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025-12-16 15:08:15</t>
+          <t>2025-12-09 16:11:28</t>
         </is>
       </c>
     </row>
@@ -518,17 +518,17 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025-12-16 14:17:46</t>
+          <t>2025-12-09 16:09:53</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>365</v>
+        <v>276</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -544,17 +544,17 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.05</v>
+        <v>-3</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2025-12-16 13:42:03</t>
+          <t>2025-12-26 11:44:24</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>365</v>
+        <v>276</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -570,17 +570,17 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.02</v>
+        <v>56</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2025-12-16 13:41:18</t>
+          <t>2025-12-26 11:08:33</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>365</v>
+        <v>276</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -596,17 +596,17 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2025-12-16 13:34:28</t>
+          <t>2025-12-26 11:07:50</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>365</v>
+        <v>276</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -622,17 +622,17 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2025-12-15 12:25:21</t>
+          <t>2025-12-26 11:06:54</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>365</v>
+        <v>276</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -648,17 +648,17 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2025-12-09 16:13:28</t>
+          <t>2025-12-26 11:05:59</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>365</v>
+        <v>276</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -674,17 +674,17 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>48</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2025-12-09 16:11:28</t>
+          <t>2025-12-26 10:53:22</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>365</v>
+        <v>276</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -700,11 +700,11 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>4.5</v>
+        <v>9</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2025-12-09 16:09:53</t>
+          <t>2025-12-26 10:52:52</t>
         </is>
       </c>
     </row>

</xml_diff>